<commit_message>
Control point 3 (#4)
* Favorite cards logic

* Added messages

* readme.md refactor

* Meta Service

* new balance analyzer

* Fixed balance analyzer

* Fixed balance anlyzer

* Fix formatting

* upd purlple card
</commit_message>
<xml_diff>
--- a/Cards.xlsx
+++ b/Cards.xlsx
@@ -70,6 +70,24 @@
     <t>Константин выложил гайд в чат — команда сыта и мотивирована.</t>
   </si>
   <si>
+    <t>Стипендия за проект</t>
+  </si>
+  <si>
+    <t>Gold</t>
+  </si>
+  <si>
+    <t>GET 6</t>
+  </si>
+  <si>
+    <t>Flux_golden-coin-with-game-controller-icon_-radiant-light_-cartoo.png</t>
+  </si>
+  <si>
+    <t>Ваш проект заметили! Первая выплата.</t>
+  </si>
+  <si>
+    <t>Получите 10 корма из банка</t>
+  </si>
+  <si>
     <t>Баланс-пати от Константина</t>
   </si>
   <si>
@@ -97,6 +115,24 @@
     <t>Спринт синхронизирован, команда в ресурсе.</t>
   </si>
   <si>
+    <t>Аудит кормов от Искандера</t>
+  </si>
+  <si>
+    <t>Red</t>
+  </si>
+  <si>
+    <t>STEAL_MONEY ALL 1</t>
+  </si>
+  <si>
+    <t>Flux_cartoon-iskander-with-magnifying-glass-inspecting-ledger_-dr.png</t>
+  </si>
+  <si>
+    <t>Искандер проверяет бюджет. Найдены излишки — изымаются.</t>
+  </si>
+  <si>
+    <t>Заберите 1 корм у всех оппонентов</t>
+  </si>
+  <si>
     <t>Грант на корм для команды</t>
   </si>
   <si>
@@ -124,6 +160,21 @@
     <t>Искандер объясняет, как корм влияет на метрики.</t>
   </si>
   <si>
+    <t>Проверка ТЗ: штраф за ошибки</t>
+  </si>
+  <si>
+    <t>STEAL_MONEY ALL 2</t>
+  </si>
+  <si>
+    <t>Flux_konstantin-with-red-pen-marking-documents_-shadows_-humorous.png</t>
+  </si>
+  <si>
+    <t>Константин нашёл несоответствия в ТЗ. Штрафуем.</t>
+  </si>
+  <si>
+    <t>Заберите 2 корма у всех оппонентов</t>
+  </si>
+  <si>
     <t>Дедлайн продлён!</t>
   </si>
   <si>
@@ -178,37 +229,19 @@
     <t>Релиз состоялся! Все получают награду.</t>
   </si>
   <si>
-    <t>Аудит кормов от Искандера</t>
-  </si>
-  <si>
-    <t>Red</t>
-  </si>
-  <si>
-    <t>STEAL_MONEY ALL 1</t>
-  </si>
-  <si>
-    <t>Flux_cartoon-iskander-with-magnifying-glass-inspecting-ledger_-dr.png</t>
-  </si>
-  <si>
-    <t>Искандер проверяет бюджет. Найдены излишки — изымаются.</t>
-  </si>
-  <si>
-    <t>Заберите 1 корм у всех оппонентов</t>
-  </si>
-  <si>
-    <t>Проверка ТЗ: штраф за ошибки</t>
-  </si>
-  <si>
-    <t>STEAL_MONEY ALL 2</t>
-  </si>
-  <si>
-    <t>Flux_konstantin-with-red-pen-marking-documents_-shadows_-humorous.png</t>
-  </si>
-  <si>
-    <t>Константин нашёл несоответствия в ТЗ. Штрафуем.</t>
-  </si>
-  <si>
-    <t>Заберите 2 корма у всех оппонентов</t>
+    <t>Грант на балансировку</t>
+  </si>
+  <si>
+    <t>GET 18</t>
+  </si>
+  <si>
+    <t>Flux_grant-document-with-golden-seal_-iskander-signing_-cartoon-s.png</t>
+  </si>
+  <si>
+    <t>Специальный грант на улучшение баланса.</t>
+  </si>
+  <si>
+    <t>Получите 20 корма из банка</t>
   </si>
   <si>
     <t>Ревизия спринта</t>
@@ -241,6 +274,24 @@
     <t>Заберите 4 корма у всех оппонентов</t>
   </si>
   <si>
+    <t>Плагиат на митапе</t>
+  </si>
+  <si>
+    <t>Purple</t>
+  </si>
+  <si>
+    <t>STEAL_CARD RANDOM</t>
+  </si>
+  <si>
+    <t>Flux_mysterious-silhouette-sneaking-a-card-from-table_-purple-neo.png</t>
+  </si>
+  <si>
+    <t>Пока все обсуждали архитектуру, вы тихонько взяли чужую идею...</t>
+  </si>
+  <si>
+    <t>Украдите случайную карту у случайного соперника</t>
+  </si>
+  <si>
     <t>Нерф баланса: забираем корм</t>
   </si>
   <si>
@@ -256,6 +307,21 @@
     <t>Заберите 5 кормов у всех оппонентов</t>
   </si>
   <si>
+    <t>Инвестиции от Искандера</t>
+  </si>
+  <si>
+    <t>GET 30</t>
+  </si>
+  <si>
+    <t>Flux_iskander-as-angel-investor-with-golden-briefcase_-sparkles_-.png</t>
+  </si>
+  <si>
+    <t>Искандер верит в ваш проект! Крупные инвестиции.</t>
+  </si>
+  <si>
+    <t>Получите 30 корма из банка</t>
+  </si>
+  <si>
     <t>Дедлайн вчера: конфискация</t>
   </si>
   <si>
@@ -329,72 +395,6 @@
   </si>
   <si>
     <t>Заберите 10 кормов у всех оппонентов</t>
-  </si>
-  <si>
-    <t>Плагиат на митапе</t>
-  </si>
-  <si>
-    <t>Purple</t>
-  </si>
-  <si>
-    <t>STEAL_CARD RANDOM</t>
-  </si>
-  <si>
-    <t>Flux_mysterious-silhouette-sneaking-a-card-from-table_-purple-neo.png</t>
-  </si>
-  <si>
-    <t>Пока все обсуждали архитектуру, вы тихонько взяли чужую идею...</t>
-  </si>
-  <si>
-    <t>Украдите случайную карту у случайного соперника</t>
-  </si>
-  <si>
-    <t>Стипендия за проект</t>
-  </si>
-  <si>
-    <t>Gold</t>
-  </si>
-  <si>
-    <t>GET 6</t>
-  </si>
-  <si>
-    <t>Flux_golden-coin-with-game-controller-icon_-radiant-light_-cartoo.png</t>
-  </si>
-  <si>
-    <t>Ваш проект заметили! Первая выплата.</t>
-  </si>
-  <si>
-    <t>Получите 10 корма из банка</t>
-  </si>
-  <si>
-    <t>Грант на балансировку</t>
-  </si>
-  <si>
-    <t>GET 18</t>
-  </si>
-  <si>
-    <t>Flux_grant-document-with-golden-seal_-iskander-signing_-cartoon-s.png</t>
-  </si>
-  <si>
-    <t>Специальный грант на улучшение баланса.</t>
-  </si>
-  <si>
-    <t>Получите 20 корма из банка</t>
-  </si>
-  <si>
-    <t>Инвестиции от Искандера</t>
-  </si>
-  <si>
-    <t>GET 30</t>
-  </si>
-  <si>
-    <t>Flux_iskander-as-angel-investor-with-golden-briefcase_-sparkles_-.png</t>
-  </si>
-  <si>
-    <t>Искандер верит в ваш проект! Крупные инвестиции.</t>
-  </si>
-  <si>
-    <t>Получите 30 корма из банка</t>
   </si>
 </sst>
 </file>
@@ -662,9 +662,9 @@
       <rgbColor rgb="ffa5a5a5"/>
       <rgbColor rgb="ff3f3f3f"/>
       <rgbColor rgb="ff56c1fe"/>
+      <rgbColor rgb="fffff056"/>
       <rgbColor rgb="ffff968c"/>
       <rgbColor rgb="ffff94ca"/>
-      <rgbColor rgb="fffff056"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -1787,641 +1787,641 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" ht="76" customHeight="1">
-      <c r="A4" t="s" s="7">
+    <row r="4" ht="100" customHeight="1">
+      <c r="A4" t="s" s="11">
         <v>19</v>
       </c>
-      <c r="B4" t="s" s="8">
-        <v>10</v>
-      </c>
-      <c r="C4" t="s" s="9">
+      <c r="B4" t="s" s="12">
         <v>20</v>
       </c>
-      <c r="D4" s="10">
-        <v>2</v>
-      </c>
-      <c r="E4" s="10">
-        <v>3</v>
-      </c>
-      <c r="F4" t="s" s="9">
+      <c r="C4" t="s" s="13">
         <v>21</v>
       </c>
-      <c r="G4" t="s" s="9">
+      <c r="D4" s="14">
+        <v>1</v>
+      </c>
+      <c r="E4" s="14">
+        <v>6</v>
+      </c>
+      <c r="F4" t="s" s="13">
         <v>22</v>
       </c>
-      <c r="H4" s="10">
-        <v>5</v>
-      </c>
-      <c r="I4" t="s" s="9">
+      <c r="G4" t="s" s="13">
         <v>23</v>
+      </c>
+      <c r="H4" s="14">
+        <v>50</v>
+      </c>
+      <c r="I4" t="s" s="13">
+        <v>24</v>
       </c>
     </row>
     <row r="5" ht="76" customHeight="1">
       <c r="A5" t="s" s="7">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B5" t="s" s="8">
         <v>10</v>
       </c>
       <c r="C5" t="s" s="9">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D5" s="10">
         <v>2</v>
       </c>
       <c r="E5" s="10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F5" t="s" s="9">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G5" t="s" s="9">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H5" s="10">
         <v>5</v>
       </c>
       <c r="I5" t="s" s="9">
-        <v>23</v>
+        <v>29</v>
       </c>
     </row>
-    <row r="6" ht="52" customHeight="1">
+    <row r="6" ht="76" customHeight="1">
       <c r="A6" t="s" s="7">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B6" t="s" s="8">
         <v>10</v>
       </c>
       <c r="C6" t="s" s="9">
+        <v>31</v>
+      </c>
+      <c r="D6" s="10">
+        <v>2</v>
+      </c>
+      <c r="E6" s="10">
+        <v>4</v>
+      </c>
+      <c r="F6" t="s" s="9">
+        <v>32</v>
+      </c>
+      <c r="G6" t="s" s="9">
+        <v>33</v>
+      </c>
+      <c r="H6" s="10">
+        <v>5</v>
+      </c>
+      <c r="I6" t="s" s="9">
         <v>29</v>
       </c>
-      <c r="D6" s="10">
-        <v>3</v>
-      </c>
-      <c r="E6" s="10">
-        <v>5</v>
-      </c>
-      <c r="F6" t="s" s="9">
+    </row>
+    <row r="7" ht="88" customHeight="1">
+      <c r="A7" t="s" s="15">
+        <v>34</v>
+      </c>
+      <c r="B7" t="s" s="16">
+        <v>35</v>
+      </c>
+      <c r="C7" t="s" s="17">
+        <v>36</v>
+      </c>
+      <c r="D7" s="18">
+        <v>2</v>
+      </c>
+      <c r="E7" s="18">
+        <v>4</v>
+      </c>
+      <c r="F7" t="s" s="17">
+        <v>37</v>
+      </c>
+      <c r="G7" t="s" s="17">
+        <v>38</v>
+      </c>
+      <c r="H7" s="18">
         <v>30</v>
       </c>
-      <c r="G6" t="s" s="9">
-        <v>31</v>
-      </c>
-      <c r="H6" s="10">
-        <v>10</v>
-      </c>
-      <c r="I6" t="s" s="9">
-        <v>32</v>
+      <c r="I7" t="s" s="17">
+        <v>39</v>
       </c>
     </row>
-    <row r="7" ht="76" customHeight="1">
-      <c r="A7" t="s" s="7">
-        <v>33</v>
-      </c>
-      <c r="B7" t="s" s="8">
-        <v>10</v>
-      </c>
-      <c r="C7" t="s" s="9">
-        <v>34</v>
-      </c>
-      <c r="D7" s="10">
-        <v>3</v>
-      </c>
-      <c r="E7" s="10">
-        <v>6</v>
-      </c>
-      <c r="F7" t="s" s="9">
-        <v>35</v>
-      </c>
-      <c r="G7" t="s" s="9">
-        <v>36</v>
-      </c>
-      <c r="H7" s="10">
-        <v>10</v>
-      </c>
-      <c r="I7" t="s" s="9">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="8" ht="88" customHeight="1">
+    <row r="8" ht="52" customHeight="1">
       <c r="A8" t="s" s="7">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B8" t="s" s="8">
         <v>10</v>
       </c>
       <c r="C8" t="s" s="9">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="D8" s="10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E8" s="10">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F8" t="s" s="9">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G8" t="s" s="9">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="H8" s="10">
         <v>10</v>
       </c>
       <c r="I8" t="s" s="9">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" ht="76" customHeight="1">
       <c r="A9" t="s" s="7">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B9" t="s" s="8">
         <v>10</v>
       </c>
       <c r="C9" t="s" s="9">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D9" s="10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E9" s="10">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F9" t="s" s="9">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="G9" t="s" s="9">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="H9" s="10">
         <v>10</v>
       </c>
       <c r="I9" t="s" s="9">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
-    <row r="10" ht="76" customHeight="1">
-      <c r="A10" t="s" s="7">
-        <v>46</v>
-      </c>
-      <c r="B10" t="s" s="8">
-        <v>10</v>
-      </c>
-      <c r="C10" t="s" s="9">
-        <v>47</v>
-      </c>
-      <c r="D10" s="10">
-        <v>5</v>
-      </c>
-      <c r="E10" s="10">
-        <v>9</v>
-      </c>
-      <c r="F10" t="s" s="9">
-        <v>48</v>
-      </c>
-      <c r="G10" t="s" s="9">
+    <row r="10" ht="88" customHeight="1">
+      <c r="A10" t="s" s="15">
         <v>49</v>
       </c>
-      <c r="H10" s="10">
-        <v>10</v>
-      </c>
-      <c r="I10" t="s" s="9">
+      <c r="B10" t="s" s="16">
+        <v>35</v>
+      </c>
+      <c r="C10" t="s" s="17">
         <v>50</v>
       </c>
+      <c r="D10" s="18">
+        <v>3</v>
+      </c>
+      <c r="E10" s="18">
+        <v>8</v>
+      </c>
+      <c r="F10" t="s" s="17">
+        <v>51</v>
+      </c>
+      <c r="G10" t="s" s="17">
+        <v>52</v>
+      </c>
+      <c r="H10" s="18">
+        <v>30</v>
+      </c>
+      <c r="I10" t="s" s="17">
+        <v>53</v>
+      </c>
     </row>
-    <row r="11" ht="64" customHeight="1">
+    <row r="11" ht="88" customHeight="1">
       <c r="A11" t="s" s="7">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B11" t="s" s="8">
         <v>10</v>
       </c>
       <c r="C11" t="s" s="9">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D11" s="10">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E11" s="10">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F11" t="s" s="9">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="G11" t="s" s="9">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H11" s="10">
         <v>10</v>
       </c>
       <c r="I11" t="s" s="9">
-        <v>50</v>
+        <v>58</v>
       </c>
     </row>
-    <row r="12" ht="88" customHeight="1">
-      <c r="A12" t="s" s="11">
-        <v>55</v>
-      </c>
-      <c r="B12" t="s" s="12">
-        <v>56</v>
-      </c>
-      <c r="C12" t="s" s="13">
-        <v>57</v>
-      </c>
-      <c r="D12" s="14">
-        <v>2</v>
-      </c>
-      <c r="E12" s="14">
+    <row r="12" ht="76" customHeight="1">
+      <c r="A12" t="s" s="7">
+        <v>59</v>
+      </c>
+      <c r="B12" t="s" s="8">
+        <v>10</v>
+      </c>
+      <c r="C12" t="s" s="9">
+        <v>60</v>
+      </c>
+      <c r="D12" s="10">
         <v>4</v>
       </c>
-      <c r="F12" t="s" s="13">
+      <c r="E12" s="10">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s" s="9">
+        <v>61</v>
+      </c>
+      <c r="G12" t="s" s="9">
+        <v>62</v>
+      </c>
+      <c r="H12" s="10">
+        <v>10</v>
+      </c>
+      <c r="I12" t="s" s="9">
         <v>58</v>
       </c>
-      <c r="G12" t="s" s="13">
-        <v>59</v>
-      </c>
-      <c r="H12" s="14">
-        <v>30</v>
-      </c>
-      <c r="I12" t="s" s="13">
-        <v>60</v>
-      </c>
     </row>
-    <row r="13" ht="88" customHeight="1">
-      <c r="A13" t="s" s="11">
-        <v>61</v>
-      </c>
-      <c r="B13" t="s" s="12">
-        <v>56</v>
-      </c>
-      <c r="C13" t="s" s="13">
-        <v>62</v>
-      </c>
-      <c r="D13" s="14">
-        <v>3</v>
-      </c>
-      <c r="E13" s="14">
-        <v>8</v>
-      </c>
-      <c r="F13" t="s" s="13">
+    <row r="13" ht="76" customHeight="1">
+      <c r="A13" t="s" s="7">
         <v>63</v>
       </c>
-      <c r="G13" t="s" s="13">
+      <c r="B13" t="s" s="8">
+        <v>10</v>
+      </c>
+      <c r="C13" t="s" s="9">
         <v>64</v>
       </c>
-      <c r="H13" s="14">
-        <v>30</v>
-      </c>
-      <c r="I13" t="s" s="13">
+      <c r="D13" s="10">
+        <v>5</v>
+      </c>
+      <c r="E13" s="10">
+        <v>9</v>
+      </c>
+      <c r="F13" t="s" s="9">
         <v>65</v>
       </c>
+      <c r="G13" t="s" s="9">
+        <v>66</v>
+      </c>
+      <c r="H13" s="10">
+        <v>10</v>
+      </c>
+      <c r="I13" t="s" s="9">
+        <v>67</v>
+      </c>
     </row>
-    <row r="14" ht="88" customHeight="1">
-      <c r="A14" t="s" s="11">
-        <v>66</v>
-      </c>
-      <c r="B14" t="s" s="12">
-        <v>56</v>
-      </c>
-      <c r="C14" t="s" s="13">
+    <row r="14" ht="64" customHeight="1">
+      <c r="A14" t="s" s="7">
+        <v>68</v>
+      </c>
+      <c r="B14" t="s" s="8">
+        <v>10</v>
+      </c>
+      <c r="C14" t="s" s="9">
+        <v>69</v>
+      </c>
+      <c r="D14" s="10">
+        <v>5</v>
+      </c>
+      <c r="E14" s="10">
+        <v>10</v>
+      </c>
+      <c r="F14" t="s" s="9">
+        <v>70</v>
+      </c>
+      <c r="G14" t="s" s="9">
+        <v>71</v>
+      </c>
+      <c r="H14" s="10">
+        <v>10</v>
+      </c>
+      <c r="I14" t="s" s="9">
         <v>67</v>
-      </c>
-      <c r="D14" s="14">
-        <v>6</v>
-      </c>
-      <c r="E14" s="14">
-        <v>12</v>
-      </c>
-      <c r="F14" t="s" s="13">
-        <v>68</v>
-      </c>
-      <c r="G14" t="s" s="13">
-        <v>69</v>
-      </c>
-      <c r="H14" s="14">
-        <v>30</v>
-      </c>
-      <c r="I14" t="s" s="13">
-        <v>70</v>
       </c>
     </row>
     <row r="15" ht="100" customHeight="1">
       <c r="A15" t="s" s="11">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B15" t="s" s="12">
-        <v>56</v>
+        <v>20</v>
       </c>
       <c r="C15" t="s" s="13">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D15" s="14">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E15" s="14">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F15" t="s" s="13">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G15" t="s" s="13">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H15" s="14">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="I15" t="s" s="13">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="16" ht="88" customHeight="1">
-      <c r="A16" t="s" s="11">
-        <v>76</v>
-      </c>
-      <c r="B16" t="s" s="12">
-        <v>56</v>
-      </c>
-      <c r="C16" t="s" s="13">
+      <c r="A16" t="s" s="15">
         <v>77</v>
       </c>
-      <c r="D16" s="14">
-        <v>10</v>
-      </c>
-      <c r="E16" s="14">
-        <v>20</v>
-      </c>
-      <c r="F16" t="s" s="13">
+      <c r="B16" t="s" s="16">
+        <v>35</v>
+      </c>
+      <c r="C16" t="s" s="17">
         <v>78</v>
       </c>
-      <c r="G16" t="s" s="13">
+      <c r="D16" s="18">
+        <v>6</v>
+      </c>
+      <c r="E16" s="18">
+        <v>12</v>
+      </c>
+      <c r="F16" t="s" s="17">
         <v>79</v>
       </c>
-      <c r="H16" s="14">
+      <c r="G16" t="s" s="17">
+        <v>80</v>
+      </c>
+      <c r="H16" s="18">
         <v>30</v>
       </c>
-      <c r="I16" t="s" s="13">
-        <v>80</v>
+      <c r="I16" t="s" s="17">
+        <v>81</v>
       </c>
     </row>
     <row r="17" ht="100" customHeight="1">
-      <c r="A17" t="s" s="11">
-        <v>81</v>
-      </c>
-      <c r="B17" t="s" s="12">
-        <v>56</v>
-      </c>
-      <c r="C17" t="s" s="13">
+      <c r="A17" t="s" s="15">
         <v>82</v>
       </c>
-      <c r="D17" s="14">
+      <c r="B17" t="s" s="16">
+        <v>35</v>
+      </c>
+      <c r="C17" t="s" s="17">
+        <v>83</v>
+      </c>
+      <c r="D17" s="18">
+        <v>8</v>
+      </c>
+      <c r="E17" s="18">
+        <v>16</v>
+      </c>
+      <c r="F17" t="s" s="17">
+        <v>84</v>
+      </c>
+      <c r="G17" t="s" s="17">
+        <v>85</v>
+      </c>
+      <c r="H17" s="18">
+        <v>30</v>
+      </c>
+      <c r="I17" t="s" s="17">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="18" ht="88" customHeight="1">
+      <c r="A18" t="s" s="19">
+        <v>87</v>
+      </c>
+      <c r="B18" t="s" s="20">
+        <v>88</v>
+      </c>
+      <c r="C18" t="s" s="21">
+        <v>89</v>
+      </c>
+      <c r="D18" s="22">
+        <v>3</v>
+      </c>
+      <c r="E18" s="22">
+        <v>200</v>
+      </c>
+      <c r="F18" t="s" s="21">
+        <v>90</v>
+      </c>
+      <c r="G18" t="s" s="21">
+        <v>91</v>
+      </c>
+      <c r="H18" s="22">
+        <v>300</v>
+      </c>
+      <c r="I18" t="s" s="21">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="19" ht="88" customHeight="1">
+      <c r="A19" t="s" s="15">
+        <v>93</v>
+      </c>
+      <c r="B19" t="s" s="16">
+        <v>35</v>
+      </c>
+      <c r="C19" t="s" s="17">
+        <v>94</v>
+      </c>
+      <c r="D19" s="18">
+        <v>10</v>
+      </c>
+      <c r="E19" s="18">
+        <v>20</v>
+      </c>
+      <c r="F19" t="s" s="17">
+        <v>95</v>
+      </c>
+      <c r="G19" t="s" s="17">
+        <v>96</v>
+      </c>
+      <c r="H19" s="18">
+        <v>30</v>
+      </c>
+      <c r="I19" t="s" s="17">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="20" ht="88" customHeight="1">
+      <c r="A20" t="s" s="11">
+        <v>98</v>
+      </c>
+      <c r="B20" t="s" s="12">
+        <v>20</v>
+      </c>
+      <c r="C20" t="s" s="13">
+        <v>99</v>
+      </c>
+      <c r="D20" s="14">
+        <v>10</v>
+      </c>
+      <c r="E20" s="14">
+        <v>30</v>
+      </c>
+      <c r="F20" t="s" s="13">
+        <v>100</v>
+      </c>
+      <c r="G20" t="s" s="13">
+        <v>101</v>
+      </c>
+      <c r="H20" s="14">
+        <v>50</v>
+      </c>
+      <c r="I20" t="s" s="13">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="21" ht="100" customHeight="1">
+      <c r="A21" t="s" s="15">
+        <v>103</v>
+      </c>
+      <c r="B21" t="s" s="16">
+        <v>35</v>
+      </c>
+      <c r="C21" t="s" s="17">
+        <v>104</v>
+      </c>
+      <c r="D21" s="18">
         <v>12</v>
       </c>
-      <c r="E17" s="14">
+      <c r="E21" s="18">
         <v>24</v>
       </c>
-      <c r="F17" t="s" s="13">
-        <v>83</v>
-      </c>
-      <c r="G17" t="s" s="13">
-        <v>84</v>
-      </c>
-      <c r="H17" s="14">
+      <c r="F21" t="s" s="17">
+        <v>105</v>
+      </c>
+      <c r="G21" t="s" s="17">
+        <v>106</v>
+      </c>
+      <c r="H21" s="18">
         <v>30</v>
       </c>
-      <c r="I17" t="s" s="13">
-        <v>85</v>
+      <c r="I21" t="s" s="17">
+        <v>107</v>
       </c>
     </row>
-    <row r="18" ht="100" customHeight="1">
-      <c r="A18" t="s" s="11">
-        <v>86</v>
-      </c>
-      <c r="B18" t="s" s="12">
-        <v>56</v>
-      </c>
-      <c r="C18" t="s" s="13">
-        <v>87</v>
-      </c>
-      <c r="D18" s="14">
+    <row r="22" ht="100" customHeight="1">
+      <c r="A22" t="s" s="15">
+        <v>108</v>
+      </c>
+      <c r="B22" t="s" s="16">
+        <v>35</v>
+      </c>
+      <c r="C22" t="s" s="17">
+        <v>109</v>
+      </c>
+      <c r="D22" s="18">
         <v>14</v>
       </c>
-      <c r="E18" s="14">
+      <c r="E22" s="18">
         <v>28</v>
       </c>
-      <c r="F18" t="s" s="13">
-        <v>88</v>
-      </c>
-      <c r="G18" t="s" s="13">
-        <v>89</v>
-      </c>
-      <c r="H18" s="14">
+      <c r="F22" t="s" s="17">
+        <v>110</v>
+      </c>
+      <c r="G22" t="s" s="17">
+        <v>111</v>
+      </c>
+      <c r="H22" s="18">
         <v>30</v>
       </c>
-      <c r="I18" t="s" s="13">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="19" ht="100" customHeight="1">
-      <c r="A19" t="s" s="11">
-        <v>91</v>
-      </c>
-      <c r="B19" t="s" s="12">
-        <v>56</v>
-      </c>
-      <c r="C19" t="s" s="13">
-        <v>92</v>
-      </c>
-      <c r="D19" s="14">
-        <v>16</v>
-      </c>
-      <c r="E19" s="14">
-        <v>32</v>
-      </c>
-      <c r="F19" t="s" s="13">
-        <v>93</v>
-      </c>
-      <c r="G19" t="s" s="13">
-        <v>94</v>
-      </c>
-      <c r="H19" s="14">
-        <v>30</v>
-      </c>
-      <c r="I19" t="s" s="13">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="20" ht="100" customHeight="1">
-      <c r="A20" t="s" s="11">
-        <v>96</v>
-      </c>
-      <c r="B20" t="s" s="12">
-        <v>56</v>
-      </c>
-      <c r="C20" t="s" s="13">
-        <v>97</v>
-      </c>
-      <c r="D20" s="14">
-        <v>18</v>
-      </c>
-      <c r="E20" s="14">
-        <v>36</v>
-      </c>
-      <c r="F20" t="s" s="13">
-        <v>98</v>
-      </c>
-      <c r="G20" t="s" s="13">
-        <v>99</v>
-      </c>
-      <c r="H20" s="14">
-        <v>30</v>
-      </c>
-      <c r="I20" t="s" s="13">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="21" ht="88" customHeight="1">
-      <c r="A21" t="s" s="11">
-        <v>101</v>
-      </c>
-      <c r="B21" t="s" s="12">
-        <v>56</v>
-      </c>
-      <c r="C21" t="s" s="13">
-        <v>102</v>
-      </c>
-      <c r="D21" s="14">
-        <v>20</v>
-      </c>
-      <c r="E21" s="14">
-        <v>40</v>
-      </c>
-      <c r="F21" t="s" s="13">
-        <v>103</v>
-      </c>
-      <c r="G21" t="s" s="13">
-        <v>104</v>
-      </c>
-      <c r="H21" s="14">
-        <v>30</v>
-      </c>
-      <c r="I21" t="s" s="13">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="22" ht="88" customHeight="1">
-      <c r="A22" t="s" s="15">
-        <v>106</v>
-      </c>
-      <c r="B22" t="s" s="16">
-        <v>107</v>
-      </c>
-      <c r="C22" t="s" s="17">
-        <v>108</v>
-      </c>
-      <c r="D22" s="18">
-        <v>8</v>
-      </c>
-      <c r="E22" s="18">
-        <v>200</v>
-      </c>
-      <c r="F22" t="s" s="17">
-        <v>109</v>
-      </c>
-      <c r="G22" t="s" s="17">
-        <v>110</v>
-      </c>
-      <c r="H22" s="18">
-        <v>15</v>
-      </c>
       <c r="I22" t="s" s="17">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="23" ht="100" customHeight="1">
-      <c r="A23" t="s" s="19">
-        <v>112</v>
-      </c>
-      <c r="B23" t="s" s="20">
+      <c r="A23" t="s" s="15">
         <v>113</v>
       </c>
-      <c r="C23" t="s" s="21">
+      <c r="B23" t="s" s="16">
+        <v>35</v>
+      </c>
+      <c r="C23" t="s" s="17">
         <v>114</v>
       </c>
-      <c r="D23" s="22">
-        <v>1</v>
-      </c>
-      <c r="E23" s="22">
-        <v>6</v>
-      </c>
-      <c r="F23" t="s" s="21">
+      <c r="D23" s="18">
+        <v>16</v>
+      </c>
+      <c r="E23" s="18">
+        <v>32</v>
+      </c>
+      <c r="F23" t="s" s="17">
         <v>115</v>
       </c>
-      <c r="G23" t="s" s="21">
+      <c r="G23" t="s" s="17">
         <v>116</v>
       </c>
-      <c r="H23" s="22">
-        <v>50</v>
-      </c>
-      <c r="I23" t="s" s="21">
+      <c r="H23" s="18">
+        <v>30</v>
+      </c>
+      <c r="I23" t="s" s="17">
         <v>117</v>
       </c>
     </row>
     <row r="24" ht="100" customHeight="1">
-      <c r="A24" t="s" s="19">
+      <c r="A24" t="s" s="15">
         <v>118</v>
       </c>
-      <c r="B24" t="s" s="20">
-        <v>113</v>
-      </c>
-      <c r="C24" t="s" s="21">
+      <c r="B24" t="s" s="16">
+        <v>35</v>
+      </c>
+      <c r="C24" t="s" s="17">
         <v>119</v>
       </c>
-      <c r="D24" s="22">
-        <v>5</v>
-      </c>
-      <c r="E24" s="22">
+      <c r="D24" s="18">
         <v>18</v>
       </c>
-      <c r="F24" t="s" s="21">
+      <c r="E24" s="18">
+        <v>36</v>
+      </c>
+      <c r="F24" t="s" s="17">
         <v>120</v>
       </c>
-      <c r="G24" t="s" s="21">
+      <c r="G24" t="s" s="17">
         <v>121</v>
       </c>
-      <c r="H24" s="22">
-        <v>50</v>
-      </c>
-      <c r="I24" t="s" s="21">
+      <c r="H24" s="18">
+        <v>30</v>
+      </c>
+      <c r="I24" t="s" s="17">
         <v>122</v>
       </c>
     </row>
     <row r="25" ht="88" customHeight="1">
-      <c r="A25" t="s" s="19">
+      <c r="A25" t="s" s="15">
         <v>123</v>
       </c>
-      <c r="B25" t="s" s="20">
-        <v>113</v>
-      </c>
-      <c r="C25" t="s" s="21">
+      <c r="B25" t="s" s="16">
+        <v>35</v>
+      </c>
+      <c r="C25" t="s" s="17">
         <v>124</v>
       </c>
-      <c r="D25" s="22">
-        <v>10</v>
-      </c>
-      <c r="E25" s="22">
+      <c r="D25" s="18">
+        <v>20</v>
+      </c>
+      <c r="E25" s="18">
+        <v>40</v>
+      </c>
+      <c r="F25" t="s" s="17">
+        <v>125</v>
+      </c>
+      <c r="G25" t="s" s="17">
+        <v>126</v>
+      </c>
+      <c r="H25" s="18">
         <v>30</v>
       </c>
-      <c r="F25" t="s" s="21">
-        <v>125</v>
-      </c>
-      <c r="G25" t="s" s="21">
-        <v>126</v>
-      </c>
-      <c r="H25" s="22">
-        <v>50</v>
-      </c>
-      <c r="I25" t="s" s="21">
+      <c r="I25" t="s" s="17">
         <v>127</v>
       </c>
     </row>

</xml_diff>